<commit_message>
2nd commit with city area added and reflected verified
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5216EFFA-887F-45DB-94D0-427151E93727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0171FB46-BFA9-4099-9945-422E1F20E0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,21 @@
 12. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
 13. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
 14. Click Submit,click,,"//button[normalize-space()='Submit']"
-15. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"</t>
+15. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+16. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+17. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
+18. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+19. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+20. Search City Area,type,triplicane,"//input[contains(@class,'p-multiselect-filter')]"
+21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'triplicane')]"
+22. Click close,click,,"//button[normalize-space()='Close']"
+23. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+25. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+26. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
+27. Open Select City Dropdown,click,,"//select[@id='cityId']"
+28. Select triplicane,click,,"//option[contains(text(),'triplicane')][last()]"
+29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'triplicane')]"</t>
   </si>
 </sst>
 </file>
@@ -463,7 +477,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="388.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
5th commit with add driver test started
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD76285-F408-4C09-94BA-F79802A3524A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252DB491-678A-4DC4-B4F2-4C36753FE6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CityArea" sheetId="1" r:id="rId1"/>
     <sheet name="CityAdmin" sheetId="2" r:id="rId2"/>
+    <sheet name="AddDriver" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -160,6 +161,27 @@
 43.Click on the "Add City Admin" button. "//button[@type='submit']"
 44. Verify Success Message,verify,,"//div[@aria-label='Info']"
 45. Verify that "Faizal" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='Faizal']"</t>
+  </si>
+  <si>
+    <t>SA_TS_3</t>
+  </si>
+  <si>
+    <t>Driver Registration</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_driver</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new driver by entering valid driver details and vehicle details.</t>
+  </si>
+  <si>
+    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"</t>
+  </si>
+  <si>
+    <t>Admin is logged in and has access to add driver module.</t>
   </si>
 </sst>
 </file>
@@ -209,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -225,6 +247,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,7 +613,7 @@
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="19.88671875" customWidth="1"/>
-    <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="3" max="3" width="25.44140625" customWidth="1"/>
     <col min="4" max="4" width="34.77734375" customWidth="1"/>
     <col min="5" max="5" width="64" customWidth="1"/>
     <col min="6" max="6" width="23.6640625" customWidth="1"/>
@@ -643,4 +669,69 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
6th commit with hidden checkbox issue fixed in add driver test
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252DB491-678A-4DC4-B4F2-4C36753FE6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C277FF-3C8C-46D0-9348-D6AA256031F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -175,13 +175,20 @@
     <t>Validate that the admin can successfully add a new driver by entering valid driver details and vehicle details.</t>
   </si>
   <si>
+    <t>Admin is logged in and has access to add driver module.</t>
+  </si>
+  <si>
     <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"</t>
-  </si>
-  <si>
-    <t>Admin is logged in and has access to add driver module.</t>
+4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+10. wait, 1000
+11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"</t>
   </si>
 </sst>
 </file>
@@ -711,7 +718,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -725,10 +732,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7th commit with url issue fixed and add driver test updated
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C277FF-3C8C-46D0-9348-D6AA256031F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2C2259-128A-4A3C-B903-CC9AB3AD82C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -188,7 +188,10 @@
 8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000
-11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"</t>
+11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+12. Enter Driver Name, type, shabeer, "//input[@placeholder='Type here' and contains(@class,'genInput')]"
+13. Enter Email, type, shabeer@gmail.com, "//div[6]//app-input[1]//div[1]//div[1]//input[1]"
+14. Enter Contact Number, type, 9937110008, "//input[@type='tel']"</t>
   </si>
 </sst>
 </file>
@@ -718,7 +721,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
10th commit with double image upload issue fixed in add driver test
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1EF4C8A-C7ED-4C2C-AE67-50413D5F9D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD555B2-120C-4D01-8BD0-2FB2B9DBF2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -189,12 +189,20 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, shabeer, "//input[@placeholder='Type here' and contains(@class,'genInput')]"
-13. Enter Email, type, shabeer@gmail.com, "//div[6]//app-input[1]//div[1]//div[1]//input[1]"
+12. Enter Driver Name, type, shabeer, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, shabeer@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
 14. Enter Contact Number, type, 9937110008, "//input[@type='tel']"
 15. wait, 1000
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
-17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"</t>
+17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Auto Option,click,,"//li[@id='pn_id_4_0']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+22. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+23. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+24. Upload Vehicle Image, uploadfile, "C:\images\vehicle.jpg", "(//input[@type='file'])[2]"
+25. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"</t>
   </si>
 </sst>
 </file>
@@ -724,7 +732,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="331.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
11th commit with seceret add driver test finished
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD555B2-120C-4D01-8BD0-2FB2B9DBF2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A05497C-C47D-4ED6-9620-7E2BE2221ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -189,9 +189,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, shabeer, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, shabeer@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 9937110008, "//input[@type='tel']"
+12. Enter Driver Name, type, shabi, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, shabi@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 9937110608, "//input[@type='tel']"
 15. wait, 1000
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -202,7 +202,16 @@
 22. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
 23. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
 24. Upload Vehicle Image, uploadfile, "C:\images\vehicle.jpg", "(//input[@type='file'])[2]"
-25. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"</t>
+25. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+29. Enter Account Holder Name, type, Shabeer, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+30. Enter Payment Email Address, type, shabeer_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+32. Click Submit, click, , "//button[contains(.,'Submit')]"
+33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+34. Wait for Toast to hide, wait, 2000</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
12th commit with xpath error fixed
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A05497C-C47D-4ED6-9620-7E2BE2221ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40FB0B4E-EDA1-4F9F-B636-EB9EABD6F450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,12 +83,27 @@
     <t>TC_CA_02_add_city_admin</t>
   </si>
   <si>
+    <t>SA_TS_3</t>
+  </si>
+  <si>
+    <t>Driver Registration</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_driver</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new driver by entering valid driver details and vehicle details.</t>
+  </si>
+  <si>
+    <t>Admin is logged in and has access to add driver module.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
 5. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-6. Click City area menu,click,,"//span[normalize-space()='City area']"
+6. Click City area menu,click,,"//span[normalize-space()='City Area']"
 7. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
 8. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
 9. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
@@ -153,29 +168,14 @@
 35.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
 36.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
 37.Click on the "Report Issue" → "FAQs" checkbox. "//div[6]//div[1]//label[6]"
-38.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer Settings']"
-39.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page Settings']"
-40.Click on the "Website Settings" → "Delivery Settings" checkbox. "//label[normalize-space()='Delivery Settings']"
-41.Click on the "Website Settings" → "Transport Settings" checkbox. "//label[normalize-space()='Transport Settings']"
+38.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+39.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+40.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[7]//div[1]//label[3]"
+41.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[7]//div[1]//label[4]"
 42.Click on the "Website Settings" → "FAQs" checkbox. "//div[7]//div[1]//label[5]"
 43.Click on the "Add City Admin" button. "//button[@type='submit']"
 44. Verify Success Message,verify,,"//div[@aria-label='Info']"
 45. Verify that "Faizal" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='Faizal']"</t>
-  </si>
-  <si>
-    <t>SA_TS_3</t>
-  </si>
-  <si>
-    <t>Driver Registration</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_driver</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new driver by entering valid driver details and vehicle details.</t>
-  </si>
-  <si>
-    <t>Admin is logged in and has access to add driver module.</t>
   </si>
   <si>
     <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
@@ -189,9 +189,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, shabi, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, shabi@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 9937110608, "//input[@type='tel']"
+12. Enter Driver Name, type, shafi, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, shafi@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 9967110608, "//input[@type='tel']"
 15. wait, 1000
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -206,7 +206,7 @@
 26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
 27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
 28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-29. Enter Account Holder Name, type, Shabeer, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+29. Enter Account Holder Name, type, Shafi, "//label[contains(.,'Account Holder Name')]/following::input[1]"
 30. Enter Payment Email Address, type, shabeer_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
 31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
@@ -615,7 +615,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -690,7 +690,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -743,22 +743,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
12th commit: Approve driver test started
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40FB0B4E-EDA1-4F9F-B636-EB9EABD6F450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715F62AD-4E99-420C-9305-734E9D075C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -96,39 +96,6 @@
   </si>
   <si>
     <t>Admin is logged in and has access to add driver module.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-6. Click City area menu,click,,"//span[normalize-space()='City Area']"
-7. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-8. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
-9. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
-10.Enter Area Name,type,triplicane,"//input[@placeholder='Area Name']"
-11. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-12. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-13. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-14. Click Submit,click,,"//button[normalize-space()='Submit']"
-15. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-16. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-17. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
-18. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-19. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-20. Search City Area,type,triplicane,"//input[contains(@class,'p-multiselect-filter')]"
-21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'triplicane')]"
-22. Click close,click,,"//button[normalize-space()='Close']"
-23. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-25. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-26. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
-27. Open Select City Dropdown,click,,"//select[@id='cityId']"
-28. Select triplicane,click,,"//option[contains(text(),'triplicane')][last()]"
-29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'triplicane')]"
-30. Click back,click,,"//button[@type='button']"
-</t>
   </si>
   <si>
     <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
@@ -178,7 +145,62 @@
 45. Verify that "Faizal" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='Faizal']"</t>
   </si>
   <si>
-    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+    <t>SA_TS_4</t>
+  </si>
+  <si>
+    <t>Driver Approval</t>
+  </si>
+  <si>
+    <t>Approve driver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+6. Click City area menu,click,,"//span[normalize-space()='City area']"
+7. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+8. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
+9. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
+10.Enter Area Name,type,triplicane,"//input[@placeholder='Area Name']"
+11. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+12. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+13. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+14. Click Submit,click,,"//button[normalize-space()='Submit']"
+15. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+16. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+17. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
+18. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+19. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+20. Search City Area,type,triplicane,"//input[contains(@class,'p-multiselect-filter')]"
+21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'triplicane')]"
+22. Click close,click,,"//button[normalize-space()='Close']"
+23. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+25. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+26. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
+27. Open Select City Dropdown,click,,"//select[@id='cityId']"
+28. Select triplicane,click,,"//option[contains(text(),'triplicane')][last()]"
+29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'triplicane')]"
+30. Click back,click,,"//button[@type='button']"
+</t>
+  </si>
+  <si>
+    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3.Click Login,click,,"//button[@type='submit']"
+4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6.Click Pending Documents,click,,"'//span[normalize-space()='Pending documents']"
+7.Filter by Name,type,rinas,"//div[contains(@class,'ag-floating-filter')]//input"
+8.Wait for Row,wait,2000,</t>
+  </si>
+  <si>
+    <t>TC_CA_04_approve_driver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
@@ -189,9 +211,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, shafi, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, shafi@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 9967110608, "//input[@type='tel']"
+12. Enter Driver Name, type, nifas, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, nifas@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 7987189608, "//input[@type='tel']"
 15. wait, 1000
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -211,7 +233,8 @@
 31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-34. Wait for Toast to hide, wait, 2000</t>
+34. Wait for Toast to hide, wait, 5000
+</t>
   </si>
 </sst>
 </file>
@@ -261,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -281,6 +304,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -615,7 +641,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -690,7 +716,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -703,7 +729,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -755,10 +781,27 @@
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
13th commit:The driver search issue ressolved Approve driver pending document
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715F62AD-4E99-420C-9305-734E9D075C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA78E12-014F-422C-A935-1F9CE40F4F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -187,16 +187,6 @@
 </t>
   </si>
   <si>
-    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3.Click Login,click,,"//button[@type='submit']"
-4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6.Click Pending Documents,click,,"'//span[normalize-space()='Pending documents']"
-7.Filter by Name,type,rinas,"//div[contains(@class,'ag-floating-filter')]//input"
-8.Wait for Row,wait,2000,</t>
-  </si>
-  <si>
     <t>TC_CA_04_approve_driver</t>
   </si>
   <si>
@@ -235,6 +225,17 @@
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 34. Wait for Toast to hide, wait, 5000
 </t>
+  </si>
+  <si>
+    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3.Click Login,click,,"//button[@type='submit']"
+4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+7.wait, 3000
+8.Filter by Name,type,rinas,"//input[@aria-label='Driver Name Filter Input']"
+8.wait,5000</t>
   </si>
 </sst>
 </file>
@@ -781,13 +782,13 @@
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -795,13 +796,13 @@
         <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
14th commit:ADD Driver and Verify driver test completed
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA78E12-014F-422C-A935-1F9CE40F4F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1EED87-DEA0-4DE0-89BD-C64B42906827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -199,12 +199,12 @@
 7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
 8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-10. wait, 1000
+10. wait, 1000,,
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, nifas, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, nifas@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 7987189608, "//input[@type='tel']"
-15. wait, 1000
+12. Enter Driver Name, type, joy, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, joy@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8530130980, "//input[@type='tel']"
+15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
 18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
@@ -223,7 +223,7 @@
 31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-34. Wait for Toast to hide, wait, 5000
+34. Wait for Toast to hide, wait, 5000,
 </t>
   </si>
   <si>
@@ -233,9 +233,30 @@
 4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
 5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-7.wait, 3000
-8.Filter by Name,type,rinas,"//input[@aria-label='Driver Name Filter Input']"
-8.wait,5000</t>
+7.wait, 3000,,
+8.Filter by Name,type,joy,"//input[@aria-label='Driver Name Filter Input']"
+9.wait,3000,,
+10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+11.wait,3000,,
+12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+13.Add Driving License,click,,"//i[@title='Edit']"
+14.wait,3000,,
+15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+17.wait,1000,,
+18.Click Submit, click, , "//button[normalize-space()='Submit']"
+19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+20.wait,2000,,
+21.Click Approve Driver,click,,"//i[@title='Approve']"
+22.wait,2000,,
+23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+24.wait,5000,,
+25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+29.Filter Approved Driver,type,joy,"//input[@aria-label='Driver Name Filter Input']"
+30.wait,3000,,</t>
   </si>
 </sst>
 </file>
@@ -788,7 +809,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="144" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
14th commit:ADD Auto Driver and Verify Auto driver test completed
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1EED87-DEA0-4DE0-89BD-C64B42906827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2373A7E3-2FD4-4262-98E8-B43331227D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CityArea" sheetId="1" r:id="rId1"/>
     <sheet name="CityAdmin" sheetId="2" r:id="rId2"/>
-    <sheet name="AddDriver" sheetId="3" r:id="rId3"/>
+    <sheet name="AddAutoDriver" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -151,9 +151,6 @@
     <t>Driver Approval</t>
   </si>
   <si>
-    <t>Approve driver</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
@@ -190,6 +187,9 @@
     <t>TC_CA_04_approve_driver</t>
   </si>
   <si>
+    <t>Validate that the added driver is created in pending documents section and upload license from this section and  approve the driver after document upload and validate that the driver is moved to approved driver section after approval.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
@@ -201,9 +201,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000,,
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, joy, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, joy@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8530130980, "//input[@type='tel']"
+12. Enter Driver Name, type, jay, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, jay@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8230000980, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -234,7 +234,7 @@
 5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
 7.wait, 3000,,
-8.Filter by Name,type,joy,"//input[@aria-label='Driver Name Filter Input']"
+8.Filter by Name,type,jay,"//input[@aria-label='Driver Name Filter Input']"
 9.wait,3000,,
 10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
 11.wait,3000,,
@@ -255,7 +255,7 @@
 26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,joy,"//input[@aria-label='Driver Name Filter Input']"
+29.Filter Approved Driver,type,jay,"//input[@aria-label='Driver Name Filter Input']"
 30.wait,3000,,</t>
   </si>
 </sst>
@@ -663,7 +663,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -817,10 +817,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
15th commit:ADD bike driver test completed
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2373A7E3-2FD4-4262-98E8-B43331227D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409991C3-5050-4806-8003-7808FE94B3F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CityArea" sheetId="1" r:id="rId1"/>
     <sheet name="CityAdmin" sheetId="2" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId3"/>
+    <sheet name="AddBikeDriver" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -84,15 +85,6 @@
   </si>
   <si>
     <t>SA_TS_3</t>
-  </si>
-  <si>
-    <t>Driver Registration</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_driver</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new driver by entering valid driver details and vehicle details.</t>
   </si>
   <si>
     <t>Admin is logged in and has access to add driver module.</t>
@@ -184,10 +176,43 @@
 </t>
   </si>
   <si>
-    <t>TC_CA_04_approve_driver</t>
-  </si>
-  <si>
-    <t>Validate that the added driver is created in pending documents section and upload license from this section and  approve the driver after document upload and validate that the driver is moved to approved driver section after approval.</t>
+    <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details.</t>
+  </si>
+  <si>
+    <t>Auto Driver Registration</t>
+  </si>
+  <si>
+    <t>Auto Driver Approval</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_bike_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_04_approve_auto_driver</t>
+  </si>
+  <si>
+    <t>Validate that the added auto driver is created in pending documents section and upload license from this section and  approve the auto driver after document upload and validate that the driver is moved to approved driver section after approval.</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new bike driver by entering valid driver details and vehicle details.</t>
+  </si>
+  <si>
+    <t>Bike Driver Registration</t>
+  </si>
+  <si>
+    <t>SA_TS_5</t>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>Validate that the added bike driver is created in pending documents section and upload license from this section and  approve the bike driver after document upload and validate that the bike driver is moved to approved driver section after approval.</t>
+  </si>
+  <si>
+    <t>TC_CA_06_approve_bike-driver</t>
   </si>
   <si>
     <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
@@ -201,9 +226,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000,,
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, jay, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, jay@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8230000980, "//input[@type='tel']"
+12. Enter Driver Name, type, jim, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, jim@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8230100980, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -234,7 +259,7 @@
 5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
 7.wait, 3000,,
-8.Filter by Name,type,jay,"//input[@aria-label='Driver Name Filter Input']"
+8.Filter by Name,type,jim,"//input[@aria-label='Driver Name Filter Input']"
 9.wait,3000,,
 10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
 11.wait,3000,,
@@ -255,7 +280,76 @@
 26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,jay,"//input[@aria-label='Driver Name Filter Input']"
+29.Filter Approved Driver,type,jim,"//input[@aria-label='Driver Name Filter Input']"
+30.wait,3000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+9.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
+10. wait, 3000,,
+11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12. Enter Driver Name, type, max, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, max@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8030010180, "//input[@type='tel']"
+15. wait, 1000,,
+16. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
+17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Scooter Option,click,,"//li[@id='pn_id_4_1']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+22. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+23. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
+24. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//input[@type='file'])[2]"
+25. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+29. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+30. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+32. Click Submit, click, , "//button[contains(.,'Submit')]"
+33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+34. Wait for Toast to hide, wait, 5000,
+</t>
+  </si>
+  <si>
+    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3.Click Login,click,,"//button[@type='submit']"
+4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+7.wait, 3000,,
+8.Filter by Name,type,max,"//input[@aria-label='Driver Name Filter Input']"
+9.wait,3000,,
+10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+11.wait,3000,,
+12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+13.Add Driving License,click,,"//i[@title='Edit']"
+14.wait,3000,,
+15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+17.wait,1000,,
+18.Click Submit, click, , "//button[normalize-space()='Submit']"
+19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+20.wait,2000,,
+21.Click Approve Driver,click,,"//i[@title='Approve']"
+22.wait,2000,,
+23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+24.wait,5000,,
+25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+29.Filter Approved Driver,type,max,"//input[@aria-label='Driver Name Filter Input']"
 30.wait,3000,,</t>
   </si>
 </sst>
@@ -663,7 +757,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -738,7 +832,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -756,7 +850,7 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="20.77734375" customWidth="1"/>
@@ -794,36 +888,118 @@
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4197A722-266E-4219-9B46-8F4D56D7D7A1}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
16th commit:ADD taxi driver test completed
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409991C3-5050-4806-8003-7808FE94B3F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2573CF0A-EDF8-4F69-8287-9CBC5E966B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CityArea" sheetId="1" r:id="rId1"/>
     <sheet name="CityAdmin" sheetId="2" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId3"/>
     <sheet name="AddBikeDriver" sheetId="4" r:id="rId4"/>
+    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -212,7 +213,28 @@
     <t>Validate that the added bike driver is created in pending documents section and upload license from this section and  approve the bike driver after document upload and validate that the bike driver is moved to approved driver section after approval.</t>
   </si>
   <si>
-    <t>TC_CA_06_approve_bike-driver</t>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>SA_TS_7</t>
+  </si>
+  <si>
+    <t>Taxi Driver Registration</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new taxi driver by entering valid driver details and vehicle details.</t>
+  </si>
+  <si>
+    <t>TC_CA_07_add_taxi_driver</t>
+  </si>
+  <si>
+    <t>Taxi Driver Approval</t>
+  </si>
+  <si>
+    <t>TC_CA_08_approve_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_06_approve_bike_driver</t>
   </si>
   <si>
     <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
@@ -226,9 +248,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000,,
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, jim, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, jim@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8230100980, "//input[@type='tel']"
+12. Enter Driver Name, type, leo, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, leo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 5230170980, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -259,7 +281,7 @@
 5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
 7.wait, 3000,,
-8.Filter by Name,type,jim,"//input[@aria-label='Driver Name Filter Input']"
+8.Filter by Name,type,leo,"//input[@aria-label='Driver Name Filter Input']"
 9.wait,3000,,
 10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
 11.wait,3000,,
@@ -280,7 +302,7 @@
 26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,jim,"//input[@aria-label='Driver Name Filter Input']"
+29.Filter Approved Driver,type,leo,"//input[@aria-label='Driver Name Filter Input']"
 30.wait,3000,,</t>
   </si>
   <si>
@@ -295,9 +317,9 @@
 9.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
 10. wait, 3000,,
 11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12. Enter Driver Name, type, max, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, max@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8030010180, "//input[@type='tel']"
+12. Enter Driver Name, type, teo, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, teo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8034510180, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -328,7 +350,7 @@
 5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
 7.wait, 3000,,
-8.Filter by Name,type,max,"//input[@aria-label='Driver Name Filter Input']"
+8.Filter by Name,type,teo,"//input[@aria-label='Driver Name Filter Input']"
 9.wait,3000,,
 10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
 11.wait,3000,,
@@ -349,7 +371,76 @@
 26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,max,"//input[@aria-label='Driver Name Filter Input']"
+29.Filter Approved Driver,type,teo,"//input[@aria-label='Driver Name Filter Input']"
+30.wait,3000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+9.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
+10. wait, 3000,,
+11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12. Enter Driver Name, type, zeo, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, zeo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, 8080010177, "//input[@type='tel']"
+15. wait, 1000,,
+16. Upload Profile Image, uploadfile, "C:\images\taxidriver.jpg", "//input[@type='file']"
+17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+22. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+23. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
+24. Upload Vehicle Image, uploadfile, "C:\images\taxi.jpg", "(//input[@type='file'])[2]"
+25. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+29. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+30. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+32. Click Submit, click, , "//button[contains(.,'Submit')]"
+33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+34. Wait for Toast to hide, wait, 5000,
+</t>
+  </si>
+  <si>
+    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
+3.Click Login,click,,"//button[@type='submit']"
+4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
+5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+7.wait, 3000,,
+8.Filter by Name,type,zeo,"//input[@aria-label='Driver Name Filter Input']"
+9.wait,3000,,
+10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+11.wait,3000,,
+12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+13.Add Driving License,click,,"//i[@title='Edit']"
+14.wait,3000,,
+15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+17.wait,1000,,
+18.Click Submit, click, , "//button[normalize-space()='Submit']"
+19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+20.wait,2000,,
+21.Click Approve Driver,click,,"//i[@title='Approve']"
+22.wait,2000,,
+23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+24.wait,5000,,
+25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+29.Filter Approved Driver,type,zeo,"//input[@aria-label='Driver Name Filter Input']"
 30.wait,3000,,</t>
   </si>
 </sst>
@@ -897,7 +988,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
@@ -917,7 +1008,7 @@
         <v>30</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -979,7 +1070,7 @@
         <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
@@ -993,13 +1084,95 @@
         <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E3" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790BFFF3-3BE5-4068-A6FF-6214BEDD72BA}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>40</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
17th commit: Add driver finished and auto data genertion implemented
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2573CF0A-EDF8-4F69-8287-9CBC5E966B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C283ABB-4CFB-4AD4-92F3-F5DEF9D38102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CityArea" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="36">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -89,6 +89,36 @@
   </si>
   <si>
     <t>Admin is logged in and has access to add driver module.</t>
+  </si>
+  <si>
+    <t>SA_TS_4</t>
+  </si>
+  <si>
+    <t>Auto Driver Registration</t>
+  </si>
+  <si>
+    <t>Bike Driver Registration</t>
+  </si>
+  <si>
+    <t>SA_TS_5</t>
+  </si>
+  <si>
+    <t>Taxi Driver Registration</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new bike driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new taxi driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list.</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_verify_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_verify_bike_driver</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
   </si>
   <si>
     <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
@@ -101,9 +131,9 @@
 8. Click Add City Admin button,click,,"//button[@class='buttonWidget']"
 9. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
 10.Click the Name field  "//input[@id='name']"
-11. Enter the Name as "Faizal" "//input[@id='name']"
+11. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
 12.Click the Email field  "//input[@id='email']"
-13.Enter the Email as " faizal@test.com " "//input[@id='email']"
+13. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
 14.Click the password field "//input[@id='password']"
 15.Enter the Password as "faizal@123". "//input[@id='password']"
 16.Click the city field  "//select[@id='cityId']"
@@ -135,13 +165,7 @@
 42.Click on the "Website Settings" → "FAQs" checkbox. "//div[7]//div[1]//label[5]"
 43.Click on the "Add City Admin" button. "//button[@type='submit']"
 44. Verify Success Message,verify,,"//div[@aria-label='Info']"
-45. Verify that "Faizal" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='Faizal']"</t>
-  </si>
-  <si>
-    <t>SA_TS_4</t>
-  </si>
-  <si>
-    <t>Driver Approval</t>
+45. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
   </si>
   <si>
     <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
@@ -153,7 +177,7 @@
 7. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
 8. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
 9. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
-10.Enter Area Name,type,triplicane,"//input[@placeholder='Area Name']"
+10. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
 11. Open Status Dropdown,click,,"//span[@aria-label='select status']"
 12. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
 13. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
@@ -163,81 +187,21 @@
 17. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
 18. Click Add Category,click,,"//button[normalize-space()='Add Category']"
 19. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-20. Search City Area,type,triplicane,"//input[contains(@class,'p-multiselect-filter')]"
-21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'triplicane')]"
+20. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
 22. Click close,click,,"//button[normalize-space()='Close']"
 23. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
 25. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
 26. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
 27. Open Select City Dropdown,click,,"//select[@id='cityId']"
-28. Select triplicane,click,,"//option[contains(text(),'triplicane')][last()]"
-29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'triplicane')]"
+28. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
 30. Click back,click,,"//button[@type='button']"
 </t>
   </si>
   <si>
-    <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details.</t>
-  </si>
-  <si>
-    <t>Auto Driver Registration</t>
-  </si>
-  <si>
-    <t>Auto Driver Approval</t>
-  </si>
-  <si>
-    <t>TC_CA_05_add_bike_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_04_approve_auto_driver</t>
-  </si>
-  <si>
-    <t>Validate that the added auto driver is created in pending documents section and upload license from this section and  approve the auto driver after document upload and validate that the driver is moved to approved driver section after approval.</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new bike driver by entering valid driver details and vehicle details.</t>
-  </si>
-  <si>
-    <t>Bike Driver Registration</t>
-  </si>
-  <si>
-    <t>SA_TS_5</t>
-  </si>
-  <si>
-    <t>SA_TS_6</t>
-  </si>
-  <si>
-    <t>Validate that the added bike driver is created in pending documents section and upload license from this section and  approve the bike driver after document upload and validate that the bike driver is moved to approved driver section after approval.</t>
-  </si>
-  <si>
-    <t>SA_TS_8</t>
-  </si>
-  <si>
-    <t>SA_TS_7</t>
-  </si>
-  <si>
-    <t>Taxi Driver Registration</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new taxi driver by entering valid driver details and vehicle details.</t>
-  </si>
-  <si>
-    <t>TC_CA_07_add_taxi_driver</t>
-  </si>
-  <si>
-    <t>Taxi Driver Approval</t>
-  </si>
-  <si>
-    <t>TC_CA_08_approve_taxi_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_06_approve_bike_driver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
@@ -248,9 +212,9 @@
 9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 10. wait, 1000,,
 11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, leo, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, leo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 5230170980, "//input[@type='tel']"
+12. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, autodriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -271,42 +235,36 @@
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 34. Wait for Toast to hide, wait, 5000,
-</t>
-  </si>
-  <si>
-    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3.Click Login,click,,"//button[@type='submit']"
-4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-7.wait, 3000,,
-8.Filter by Name,type,leo,"//input[@aria-label='Driver Name Filter Input']"
-9.wait,3000,,
-10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-11.wait,3000,,
-12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-13.Add Driving License,click,,"//i[@title='Edit']"
-14.wait,3000,,
-15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-17.wait,1000,,
-18.Click Submit, click, , "//button[normalize-space()='Submit']"
-19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-20.wait,2000,,
-21.Click Approve Driver,click,,"//i[@title='Approve']"
-22.wait,2000,,
-23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-24.wait,5000,,
-25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,leo,"//input[@aria-label='Driver Name Filter Input']"
-30.wait,3000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+38.wait, 3000,,
+39.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+40.wait,3000,,
+41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+42.wait,3000,,
+43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+44.Add Driving License,click,,"//i[@title='Edit']"
+45.wait,3000,,
+46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+48.wait,1000,,
+49.Click Submit, click, , "//button[normalize-space()='Submit']"
+50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+51.wait,2000,,
+52.Click Approve Driver,click,,"//i[@title='Approve']"
+53.wait,2000,,
+54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+55.wait,5000,,
+56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+60.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+61.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
@@ -317,9 +275,9 @@
 9.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
 10. wait, 3000,,
 11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12. Enter Driver Name, type, teo, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, teo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8034510180, "//input[@type='tel']"
+12. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, bikedriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -340,42 +298,36 @@
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 34. Wait for Toast to hide, wait, 5000,
-</t>
-  </si>
-  <si>
-    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3.Click Login,click,,"//button[@type='submit']"
-4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-7.wait, 3000,,
-8.Filter by Name,type,teo,"//input[@aria-label='Driver Name Filter Input']"
-9.wait,3000,,
-10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-11.wait,3000,,
-12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-13.Add Driving License,click,,"//i[@title='Edit']"
-14.wait,3000,,
-15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-17.wait,1000,,
-18.Click Submit, click, , "//button[normalize-space()='Submit']"
-19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-20.wait,2000,,
-21.Click Approve Driver,click,,"//i[@title='Approve']"
-22.wait,2000,,
-23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-24.wait,5000,,
-25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,teo,"//input[@aria-label='Driver Name Filter Input']"
-30.wait,3000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
+35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+38.wait, 3000,,
+39.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+40.wait,3000,,
+41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+42.wait,3000,,
+43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+44.Add Driving License,click,,"//i[@title='Edit']"
+45.wait,3000,,
+46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+48.wait,1000,,
+49.Click Submit, click, , "//button[normalize-space()='Submit']"
+50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+51.wait,2000,,
+52.Click Approve Driver,click,,"//i[@title='Approve']"
+53.wait,2000,,
+54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+55.wait,5000,,
+56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+60.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+61.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
@@ -386,9 +338,9 @@
 9.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
 10. wait, 3000,,
 11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12. Enter Driver Name, type, zeo, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, zeo@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, 8080010177, "//input[@type='tel']"
+12. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
+13. Enter Email, type, taxidriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 15. wait, 1000,,
 16. Upload Profile Image, uploadfile, "C:\images\taxidriver.jpg", "//input[@type='file']"
 17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
@@ -409,39 +361,36 @@
 32. Click Submit, click, , "//button[contains(.,'Submit')]"
 33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 34. Wait for Toast to hide, wait, 5000,
-</t>
-  </si>
-  <si>
-    <t>1.Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2.Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3.Click Login,click,,"//button[@type='submit']"
-4.Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-7.wait, 3000,,
-8.Filter by Name,type,zeo,"//input[@aria-label='Driver Name Filter Input']"
-9.wait,3000,,
-10.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-11.wait,3000,,
-12. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-13.Add Driving License,click,,"//i[@title='Edit']"
-14.wait,3000,,
-15.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-16.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-17.wait,1000,,
-18.Click Submit, click, , "//button[normalize-space()='Submit']"
-19.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-20.wait,2000,,
-21.Click Approve Driver,click,,"//i[@title='Approve']"
-22.wait,2000,,
-23.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-24.wait,5000,,
-25.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-26.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-27.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-28.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-29.Filter Approved Driver,type,zeo,"//input[@aria-label='Driver Name Filter Input']"
-30.wait,3000,,</t>
+35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+38.wait, 3000,,
+39.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+40.wait,3000,,
+41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+42.wait,3000,,
+43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+44.Add Driving License,click,,"//i[@title='Edit']"
+45.wait,3000,,
+46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+48.wait,1000,,
+49.Click Submit, click, , "//button[normalize-space()='Submit']"
+50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+51.wait,2000,,
+52.Click Approve Driver,click,,"//i[@title='Approve']"
+53.wait,2000,,
+54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+55.wait,5000,,
+56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+60.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+61.wait,3000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_verify_auto_driver</t>
   </si>
 </sst>
 </file>
@@ -848,7 +797,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -923,7 +872,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -941,7 +890,7 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="27.77734375" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="20.77734375" customWidth="1"/>
@@ -979,37 +928,27 @@
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>45</v>
-      </c>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1023,7 +962,7 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="20.77734375" customWidth="1"/>
@@ -1058,40 +997,30 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>47</v>
-      </c>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1105,7 +1034,7 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" customWidth="1"/>
+    <col min="3" max="3" width="29.5546875" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="20.77734375" customWidth="1"/>
@@ -1140,40 +1069,30 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>49</v>
-      </c>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
18th commit: Single login implemtented for abc
</commit_message>
<xml_diff>
--- a/testingwe13.xlsx
+++ b/testingwe13.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C283ABB-4CFB-4AD4-92F3-F5DEF9D38102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396FA2F2-D065-4D19-AA0B-9EBA181C0AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="CityArea" sheetId="1" r:id="rId1"/>
-    <sheet name="CityAdmin" sheetId="2" r:id="rId2"/>
-    <sheet name="AddAutoDriver" sheetId="3" r:id="rId3"/>
-    <sheet name="AddBikeDriver" sheetId="4" r:id="rId4"/>
-    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId5"/>
+    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
+    <sheet name="CityArea" sheetId="1" r:id="rId2"/>
+    <sheet name="CityAdmin" sheetId="2" r:id="rId3"/>
+    <sheet name="AddAutoDriver" sheetId="3" r:id="rId4"/>
+    <sheet name="AddBikeDriver" sheetId="4" r:id="rId5"/>
+    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="40">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -121,276 +122,276 @@
     <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
   </si>
   <si>
-    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-6. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-7. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-8. Click Add City Admin button,click,,"//button[@class='buttonWidget']"
-9. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-10.Click the Name field  "//input[@id='name']"
-11. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-12.Click the Email field  "//input[@id='email']"
-13. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-14.Click the password field "//input[@id='password']"
-15.Enter the Password as "faizal@123". "//input[@id='password']"
-16.Click the city field  "//select[@id='cityId']"
-17.Select the City as "triplicane" from the dropdown "//select[@id='cityId']"
-18. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-19.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-20.Click on the "Customers" → "Verified Customers"checkbox. "//div[3]//div[1]//div[1]//label[2]"
-21.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-22.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-23.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-24.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-25.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-26.Click on the "Drivers" → "Approved Drivers" checkbox. "//body//app-root//div[3]//div[3]//div[1]//label[2]"
-27.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-28.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-29.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-30.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-31.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-32.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-33.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-34.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-35.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-36.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-37.Click on the "Report Issue" → "FAQs" checkbox. "//div[6]//div[1]//label[6]"
-38.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-39.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-40.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[7]//div[1]//label[3]"
-41.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[7]//div[1]//label[4]"
-42.Click on the "Website Settings" → "FAQs" checkbox. "//div[7]//div[1]//label[5]"
-43.Click on the "Add City Admin" button. "//button[@type='submit']"
-44. Verify Success Message,verify,,"//div[@aria-label='Info']"
-45. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
+    <t>TC_CA_03_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>SA_TS_0</t>
+  </si>
+  <si>
+    <t>TC_CA_00_City_admin_login</t>
+  </si>
+  <si>
+    <t>Verify that an  super admin can login with the provided credentials</t>
   </si>
   <si>
     <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
 2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
 3. Click Login,click,,"//button[@type='submit']"
 4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-6. Click City area menu,click,,"//span[normalize-space()='City area']"
-7. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-8. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
-9. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
-10. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-11. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-12. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-13. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-14. Click Submit,click,,"//button[normalize-space()='Submit']"
-15. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-16. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-17. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
-18. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-19. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-20. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-21. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-22. Click close,click,,"//button[normalize-space()='Close']"
-23. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-25. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-26. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
-27. Open Select City Dropdown,click,,"//select[@id='cityId']"
-28. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-30. Click back,click,,"//button[@type='button']"
 </t>
   </si>
   <si>
-    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
-8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-9.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-10. wait, 1000,,
-11. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-12. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, autodriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-15. wait, 1000,,
-16. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
-17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Auto Option,click,,"//li[@id='pn_id_4_0']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-22. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-23. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-24. Upload Vehicle Image, uploadfile, "C:\images\vehicle.jpg", "(//input[@type='file'])[2]"
-25. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-29. Enter Account Holder Name, type, Shafi, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-30. Enter Payment Email Address, type, shabeer_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-32. Click Submit, click, , "//button[contains(.,'Submit')]"
-33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-34. Wait for Toast to hide, wait, 5000,
-35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-38.wait, 3000,,
-39.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-40.wait,3000,,
-41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
+5. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+26. Click back,click,,"//button[@type='button']"
+</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7. wait, 1000,,
+8. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+9. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, autodriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+12. wait, 1000,,
+13. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
+14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+16.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+18.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+19. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+20. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+21. Upload Vehicle Image, uploadfile, "C:\images\vehicle.jpg", "(//input[@type='file'])[2]"
+22. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26. Enter Account Holder Name, type, Shafi, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, shabeer_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 5000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+35.wait, 3000,,
+36.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+37.wait,3000,,
+38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+39.wait,3000,,
+40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+41.Add Driving License,click,,"//i[@title='Edit']"
 42.wait,3000,,
-43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-44.Add Driving License,click,,"//i[@title='Edit']"
-45.wait,3000,,
-46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-48.wait,1000,,
-49.Click Submit, click, , "//button[normalize-space()='Submit']"
-50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-51.wait,2000,,
-52.Click Approve Driver,click,,"//i[@title='Approve']"
-53.wait,2000,,
-54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-55.wait,5000,,
-56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-60.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-61.wait,3000,,</t>
-  </si>
-  <si>
-    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
-8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-9.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
-10. wait, 3000,,
-11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, bikedriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-15. wait, 1000,,
-16. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
-17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Scooter Option,click,,"//li[@id='pn_id_4_1']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-22. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-23. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
-24. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//input[@type='file'])[2]"
-25. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-29. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-30. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-32. Click Submit, click, , "//button[contains(.,'Submit')]"
-33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-34. Wait for Toast to hide, wait, 5000,
-35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-38.wait, 3000,,
-39.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-40.wait,3000,,
-41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+45.wait,1000,,
+46.Click Submit, click, , "//button[normalize-space()='Submit']"
+47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+48.wait,2000,,
+49.Click Approve Driver,click,,"//i[@title='Approve']"
+50.wait,2000,,
+51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+52.wait,5000,,
+53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+57.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+58.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+5. Click Add City Admin button,click,,"//button[@class='buttonWidget']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Click the Name field  "//input[@id='name']"
+8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
+9.Click the Email field  "//input[@id='email']"
+10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
+11.Click the password field "//input[@id='password']"
+12.Enter the Password as "faizal@123". "//input[@id='password']"
+13.Click the city field  "//select[@id='cityId']"
+14.Select the City as "triplicane" from the dropdown "//select[@id='cityId']"
+15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
+17.Click on the "Customers" → "Verified Customers"checkbox. "//div[3]//div[1]//div[1]//label[2]"
+18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
+19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
+20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
+21.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+22.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+23.Click on the "Drivers" → "Approved Drivers" checkbox. "//body//app-root//div[3]//div[3]//div[1]//label[2]"
+24.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+25.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+26.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+27.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+29.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+30.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+31.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+33.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+34.Click on the "Report Issue" → "FAQs" checkbox. "//div[6]//div[1]//label[6]"
+35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+36.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+37.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[7]//div[1]//label[3]"
+38.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[7]//div[1]//label[4]"
+39.Click on the "Website Settings" → "FAQs" checkbox. "//div[7]//div[1]//label[5]"
+40.Click on the "Add City Admin" button. "//button[@type='submit']"
+41. Verify Success Message,verify,,"//div[@aria-label='Info']"
 42.wait,3000,,
-43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-44.Add Driving License,click,,"//i[@title='Edit']"
-45.wait,3000,,
-46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-48.wait,1000,,
-49.Click Submit, click, , "//button[normalize-space()='Submit']"
-50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-51.wait,2000,,
-52.Click Approve Driver,click,,"//i[@title='Approve']"
-53.wait,2000,,
-54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-55.wait,5000,,
-56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-60.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-61.wait,3000,,</t>
-  </si>
-  <si>
-    <t>1. Enter Email,type,super_admin@gmail.com,"//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321,"//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-5. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-6. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-7. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
-8.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-9.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
-10. wait, 3000,,
-11. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
-13. Enter Email, type, taxidriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-14. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-15. wait, 1000,,
-16. Upload Profile Image, uploadfile, "C:\images\taxidriver.jpg", "//input[@type='file']"
-17. Select Male Gender, click, , "//mat-radio-button[@id='mat-radio-2']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-22. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-23. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
-24. Upload Vehicle Image, uploadfile, "C:\images\taxi.jpg", "(//input[@type='file'])[2]"
-25. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-26. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-27. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-28. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-29. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-30. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-31. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-32. Click Submit, click, , "//button[contains(.,'Submit')]"
-33. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-34. Wait for Toast to hide, wait, 5000,
-35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-36.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-37.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-38.wait, 3000,,
-39.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-40.wait,3000,,
-41.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+42. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
+7. wait, 3000,,
+8. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+9. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, bikedriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+12. wait, 1000,,
+13. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
+14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+16.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
+17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+18.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+20. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
+21. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//input[@type='file'])[2]"
+22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 5000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+35.wait, 3000,,
+36.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+37.wait,3000,,
+38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+39.wait,3000,,
+40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+41.Add Driving License,click,,"//i[@title='Edit']"
 42.wait,3000,,
-43. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-44.Add Driving License,click,,"//i[@title='Edit']"
-45.wait,3000,,
-46.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
-47.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-48.wait,1000,,
-49.Click Submit, click, , "//button[normalize-space()='Submit']"
-50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-51.wait,2000,,
-52.Click Approve Driver,click,,"//i[@title='Approve']"
-53.wait,2000,,
-54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-55.wait,5000,,
-56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-59.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-60.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-61.wait,3000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_verify_auto_driver</t>
+43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+45.wait,1000,,
+46.Click Submit, click, , "//button[normalize-space()='Submit']"
+47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+48.wait,2000,,
+49.Click Approve Driver,click,,"//i[@title='Approve']"
+50.wait,2000,,
+51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+52.wait,5000,,
+53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+57.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+58.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
+7. wait, 3000,,
+8. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+9. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, taxidriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+12. wait, 1000,,
+13. Upload Profile Image, uploadfile, "C:\images\taxidriver.jpg", "//input[@type='file']"
+14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+16.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
+17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+18.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+20. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
+21. Upload Vehicle Image, uploadfile, "C:\images\taxi.jpg", "(//input[@type='file'])[2]"
+22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 5000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+35.wait, 3000,,
+36.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+37.wait,3000,,
+38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+39.wait,3000,,
+40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+41.Add Driving License,click,,"//i[@title='Edit']"
+42.wait,3000,,
+43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+45.wait,1000,,
+46.Click Submit, click, , "//button[normalize-space()='Submit']"
+47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+48.wait,2000,,
+49.Click Approve Driver,click,,"//i[@title='Approve']"
+50.wait,2000,,
+51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+52.wait,5000,,
+53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+57.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+58.wait,3000,,</t>
   </si>
 </sst>
 </file>
@@ -743,6 +744,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -797,7 +874,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -818,7 +895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -872,7 +949,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -883,7 +960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -931,13 +1008,13 @@
         <v>21</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
@@ -955,7 +1032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4197A722-266E-4219-9B46-8F4D56D7D7A1}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1009,7 +1086,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
@@ -1027,7 +1104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790BFFF3-3BE5-4068-A6FF-6214BEDD72BA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1081,7 +1158,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>

</xml_diff>